<commit_message>
added eastern sand darter (AMPE-1)
tweaked excel
</commit_message>
<xml_diff>
--- a/Objective 2/Data/Study_metadata.xlsx
+++ b/Objective 2/Data/Study_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://buckeyemailosu-my.sharepoint.com/personal/mccall_257_buckeyemail_osu_edu/Documents/Spring_2026/Landgen_DGS/DGS-Patterns-of-Fish-Diversity/DGS-Patterns-of-Fish-Diversity/Objective 2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{D0FE9348-49AB-D84F-A51D-D9F26EF9DB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BE76021-D73A-3643-B443-B6488BA68946}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{D0FE9348-49AB-D84F-A51D-D9F26EF9DB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54CB0323-5C0A-1C42-9D96-BFB5647E3EFB}"/>
   <bookViews>
     <workbookView xWindow="2480" yWindow="-21100" windowWidth="27640" windowHeight="16180" xr2:uid="{BFE04C59-CE9B-744B-B3FF-DA35D679F80E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Study_ID</t>
   </si>
@@ -60,6 +60,15 @@
   </si>
   <si>
     <t>NA. Thesis</t>
+  </si>
+  <si>
+    <t>Spp</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>Leuciscidae</t>
   </si>
 </sst>
 </file>
@@ -434,39 +443,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B3D815D-5E91-F643-AF9A-1DD227761228}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="2" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.83203125" style="1"/>
+    <col min="1" max="3" width="10.83203125" style="1"/>
+    <col min="4" max="4" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added ~10 spp data for obj 2
fst and site locations are in each spp data folder
</commit_message>
<xml_diff>
--- a/Objective 2/Data/Study_metadata.xlsx
+++ b/Objective 2/Data/Study_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://buckeyemailosu-my.sharepoint.com/personal/mccall_257_buckeyemail_osu_edu/Documents/Spring_2026/Landgen_DGS/DGS-Patterns-of-Fish-Diversity/DGS-Patterns-of-Fish-Diversity/Objective 2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{D0FE9348-49AB-D84F-A51D-D9F26EF9DB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BF54F36-4523-FD49-AFBE-A9F0F0AC8105}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="8_{D0FE9348-49AB-D84F-A51D-D9F26EF9DB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F16B5851-4C7A-7946-9984-6463974A6C6D}"/>
   <bookViews>
-    <workbookView xWindow="2480" yWindow="-21100" windowWidth="27640" windowHeight="16180" xr2:uid="{BFE04C59-CE9B-744B-B3FF-DA35D679F80E}"/>
+    <workbookView xWindow="5380" yWindow="-21100" windowWidth="27640" windowHeight="16180" xr2:uid="{BFE04C59-CE9B-744B-B3FF-DA35D679F80E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="56">
   <si>
     <t>Study_ID</t>
   </si>
@@ -108,13 +108,109 @@
   </si>
   <si>
     <t>NA. thesis</t>
+  </si>
+  <si>
+    <t>CARI-1</t>
+  </si>
+  <si>
+    <t>Klamath Smallscale Sucker</t>
+  </si>
+  <si>
+    <t>Catostomus rimiculus</t>
+  </si>
+  <si>
+    <t>Catostomidae</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/s10592-024-01651-5</t>
+  </si>
+  <si>
+    <t>ETCA-1</t>
+  </si>
+  <si>
+    <t>Rainbow Darter</t>
+  </si>
+  <si>
+    <t>Etheostoma caeruleum</t>
+  </si>
+  <si>
+    <t>Percidae</t>
+  </si>
+  <si>
+    <t>ETCA-2</t>
+  </si>
+  <si>
+    <t>https://scholarworks.uni.edu/etd/2455</t>
+  </si>
+  <si>
+    <t>DOI: 10.1002/ece3.8422</t>
+  </si>
+  <si>
+    <t>ETNI-1</t>
+  </si>
+  <si>
+    <t>Johnny Darter</t>
+  </si>
+  <si>
+    <t>Etheostoma nigrum</t>
+  </si>
+  <si>
+    <t>Tessellated darters</t>
+  </si>
+  <si>
+    <t>ETOL-1</t>
+  </si>
+  <si>
+    <t>Etheostoma olmstedi</t>
+  </si>
+  <si>
+    <t>Yazoo Darter</t>
+  </si>
+  <si>
+    <t>Etheostoma Raneyi</t>
+  </si>
+  <si>
+    <t>ETRA-1</t>
+  </si>
+  <si>
+    <t>Kentucky Arrow Darter</t>
+  </si>
+  <si>
+    <t>Etheostoma sagitta spilotum)</t>
+  </si>
+  <si>
+    <t>ETSA-1</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/s10592-019-01188-y</t>
+  </si>
+  <si>
+    <t>FUNO-1</t>
+  </si>
+  <si>
+    <t>FUOL-1</t>
+  </si>
+  <si>
+    <t>Fundulus notatus</t>
+  </si>
+  <si>
+    <t>Fundulus olivaceus</t>
+  </si>
+  <si>
+    <t>Blackstripe topminnow</t>
+  </si>
+  <si>
+    <t>Blackspotted topminnow,</t>
+  </si>
+  <si>
+    <t>Fundulidae</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -125,6 +221,21 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -146,17 +257,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -489,111 +605,308 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B3D815D-5E91-F643-AF9A-1DD227761228}">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="2" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="1"/>
-    <col min="7" max="7" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" style="2"/>
+    <col min="2" max="2" width="23.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" style="2"/>
+    <col min="7" max="7" width="38.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="F3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="E4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>23</v>
       </c>
     </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{653DA17D-ECDD-E64B-9D03-571B884756B4}"/>
+    <hyperlink ref="G7" r:id="rId2" xr:uid="{31E17336-E2E8-2F49-8F8B-E195A587BAA9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added creek chub and brook trout
yeet
</commit_message>
<xml_diff>
--- a/Objective 2/Data/Study_metadata.xlsx
+++ b/Objective 2/Data/Study_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://buckeyemailosu-my.sharepoint.com/personal/mccall_257_buckeyemail_osu_edu/Documents/Spring_2026/Landgen_DGS/DGS-Patterns-of-Fish-Diversity/DGS-Patterns-of-Fish-Diversity/Objective 2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="164" documentId="8_{D0FE9348-49AB-D84F-A51D-D9F26EF9DB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E902859D-3DFA-F749-949C-47800BDC5C67}"/>
+  <xr:revisionPtr revIDLastSave="181" documentId="8_{D0FE9348-49AB-D84F-A51D-D9F26EF9DB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCA00543-780F-1643-91AC-1803C0BF732A}"/>
   <bookViews>
     <workbookView xWindow="13340" yWindow="-21100" windowWidth="20620" windowHeight="16180" xr2:uid="{BFE04C59-CE9B-744B-B3FF-DA35D679F80E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="92">
   <si>
     <t>Study_ID</t>
   </si>
@@ -293,7 +293,25 @@
     <t>Bull trout</t>
   </si>
   <si>
-    <t>Salevlinus confluentus</t>
+    <t>SAFO-1</t>
+  </si>
+  <si>
+    <t>Brook Trout</t>
+  </si>
+  <si>
+    <t>Salevlinus fontinalis</t>
+  </si>
+  <si>
+    <t>Salvelinus confluentus</t>
+  </si>
+  <si>
+    <t>SEAT-1</t>
+  </si>
+  <si>
+    <t>Creek Chub</t>
+  </si>
+  <si>
+    <t>Campostoma anomalum</t>
   </si>
 </sst>
 </file>
@@ -698,7 +716,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B3D815D-5E91-F643-AF9A-1DD227761228}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="2"/>
@@ -764,8 +782,8 @@
       <c r="B3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>18</v>
+      <c r="C3" s="4" t="s">
+        <v>91</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
@@ -1149,7 +1167,7 @@
         <v>84</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>79</v>
@@ -1158,6 +1176,46 @@
         <v>5</v>
       </c>
       <c r="F21" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A22" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A23" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>